<commit_message>
Inicio de carga DW
</commit_message>
<xml_diff>
--- a/excel/compras.xlsx
+++ b/excel/compras.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\progs\BI\BI_Farmacias\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{995D249E-B5AA-4C17-A1F7-3D52B7F7D91B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC5E3A4F-AC0C-424D-972E-DA090193DCB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29730" yWindow="0" windowWidth="21720" windowHeight="15480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="390" yWindow="390" windowWidth="21720" windowHeight="15480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Compras_2025_2026" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16785" uniqueCount="3011">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16785" uniqueCount="3014">
   <si>
     <t>id_compra</t>
   </si>
@@ -9057,6 +9057,15 @@
   </si>
   <si>
     <t>VAALLE</t>
+  </si>
+  <si>
+    <t>PARCIAL</t>
+  </si>
+  <si>
+    <t>RECHAZADO</t>
+  </si>
+  <si>
+    <t>CANCELADO</t>
   </si>
 </sst>
 </file>
@@ -11235,7 +11244,7 @@
         <v>45670</v>
       </c>
       <c r="AB11" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC11" t="s">
         <v>46</v>
@@ -11324,7 +11333,7 @@
         <v>45671</v>
       </c>
       <c r="AB12" t="s">
-        <v>45</v>
+        <v>3012</v>
       </c>
       <c r="AC12" t="s">
         <v>46</v>
@@ -11591,7 +11600,7 @@
         <v>45673</v>
       </c>
       <c r="AB15" t="s">
-        <v>45</v>
+        <v>3013</v>
       </c>
       <c r="AC15" t="s">
         <v>46</v>
@@ -11947,7 +11956,7 @@
         <v>45678</v>
       </c>
       <c r="AB19" t="s">
-        <v>45</v>
+        <v>2894</v>
       </c>
       <c r="AC19" t="s">
         <v>46</v>
@@ -12125,7 +12134,7 @@
         <v>45678</v>
       </c>
       <c r="AB21" t="s">
-        <v>45</v>
+        <v>3013</v>
       </c>
       <c r="AC21" t="s">
         <v>46</v>
@@ -12214,7 +12223,7 @@
         <v>45676</v>
       </c>
       <c r="AB22" t="s">
-        <v>45</v>
+        <v>3012</v>
       </c>
       <c r="AC22" t="s">
         <v>46</v>
@@ -12303,7 +12312,7 @@
         <v>45682</v>
       </c>
       <c r="AB23" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC23" t="s">
         <v>46</v>
@@ -12570,7 +12579,7 @@
         <v>45683</v>
       </c>
       <c r="AB26" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC26" t="s">
         <v>46</v>
@@ -12837,7 +12846,7 @@
         <v>45687</v>
       </c>
       <c r="AB29" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC29" t="s">
         <v>46</v>
@@ -12926,7 +12935,7 @@
         <v>45683</v>
       </c>
       <c r="AB30" t="s">
-        <v>45</v>
+        <v>3012</v>
       </c>
       <c r="AC30" t="s">
         <v>46</v>
@@ -13193,7 +13202,7 @@
         <v>45688</v>
       </c>
       <c r="AB33" t="s">
-        <v>45</v>
+        <v>3013</v>
       </c>
       <c r="AC33" t="s">
         <v>46</v>
@@ -13549,7 +13558,7 @@
         <v>45691</v>
       </c>
       <c r="AB37" t="s">
-        <v>45</v>
+        <v>2894</v>
       </c>
       <c r="AC37" t="s">
         <v>46</v>
@@ -13727,7 +13736,7 @@
         <v>45695</v>
       </c>
       <c r="AB39" t="s">
-        <v>45</v>
+        <v>3013</v>
       </c>
       <c r="AC39" t="s">
         <v>46</v>
@@ -13816,7 +13825,7 @@
         <v>45691</v>
       </c>
       <c r="AB40" t="s">
-        <v>45</v>
+        <v>3012</v>
       </c>
       <c r="AC40" t="s">
         <v>46</v>
@@ -13905,7 +13914,7 @@
         <v>45697</v>
       </c>
       <c r="AB41" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC41" t="s">
         <v>46</v>
@@ -14172,7 +14181,7 @@
         <v>45694</v>
       </c>
       <c r="AB44" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC44" t="s">
         <v>46</v>
@@ -14261,7 +14270,7 @@
         <v>45700</v>
       </c>
       <c r="AB45" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC45" t="s">
         <v>46</v>
@@ -14350,7 +14359,7 @@
         <v>45700</v>
       </c>
       <c r="AB46" t="s">
-        <v>45</v>
+        <v>3012</v>
       </c>
       <c r="AC46" t="s">
         <v>46</v>
@@ -14617,7 +14626,7 @@
         <v>45701</v>
       </c>
       <c r="AB49" t="s">
-        <v>45</v>
+        <v>3013</v>
       </c>
       <c r="AC49" t="s">
         <v>46</v>
@@ -14973,7 +14982,7 @@
         <v>45705</v>
       </c>
       <c r="AB53" t="s">
-        <v>45</v>
+        <v>2894</v>
       </c>
       <c r="AC53" t="s">
         <v>46</v>
@@ -15151,7 +15160,7 @@
         <v>45706</v>
       </c>
       <c r="AB55" t="s">
-        <v>45</v>
+        <v>3013</v>
       </c>
       <c r="AC55" t="s">
         <v>46</v>
@@ -15240,7 +15249,7 @@
         <v>45704</v>
       </c>
       <c r="AB56" t="s">
-        <v>45</v>
+        <v>3012</v>
       </c>
       <c r="AC56" t="s">
         <v>46</v>
@@ -15329,7 +15338,7 @@
         <v>45710</v>
       </c>
       <c r="AB57" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC57" t="s">
         <v>46</v>
@@ -15596,7 +15605,7 @@
         <v>45711</v>
       </c>
       <c r="AB60" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC60" t="s">
         <v>46</v>
@@ -16219,7 +16228,7 @@
         <v>45718</v>
       </c>
       <c r="AB67" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC67" t="s">
         <v>46</v>
@@ -16308,7 +16317,7 @@
         <v>45718</v>
       </c>
       <c r="AB68" t="s">
-        <v>45</v>
+        <v>3012</v>
       </c>
       <c r="AC68" t="s">
         <v>46</v>
@@ -16575,7 +16584,7 @@
         <v>45720</v>
       </c>
       <c r="AB71" t="s">
-        <v>45</v>
+        <v>3013</v>
       </c>
       <c r="AC71" t="s">
         <v>46</v>
@@ -16931,7 +16940,7 @@
         <v>45721</v>
       </c>
       <c r="AB75" t="s">
-        <v>45</v>
+        <v>2894</v>
       </c>
       <c r="AC75" t="s">
         <v>46</v>
@@ -17109,7 +17118,7 @@
         <v>45726</v>
       </c>
       <c r="AB77" t="s">
-        <v>45</v>
+        <v>3013</v>
       </c>
       <c r="AC77" t="s">
         <v>46</v>
@@ -17198,7 +17207,7 @@
         <v>45722</v>
       </c>
       <c r="AB78" t="s">
-        <v>45</v>
+        <v>3012</v>
       </c>
       <c r="AC78" t="s">
         <v>46</v>
@@ -17287,7 +17296,7 @@
         <v>45728</v>
       </c>
       <c r="AB79" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC79" t="s">
         <v>46</v>
@@ -17554,7 +17563,7 @@
         <v>45725</v>
       </c>
       <c r="AB82" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC82" t="s">
         <v>46</v>
@@ -18711,7 +18720,7 @@
         <v>45741</v>
       </c>
       <c r="AB95" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC95" t="s">
         <v>46</v>
@@ -18800,7 +18809,7 @@
         <v>45741</v>
       </c>
       <c r="AB96" t="s">
-        <v>45</v>
+        <v>3012</v>
       </c>
       <c r="AC96" t="s">
         <v>46</v>
@@ -19067,7 +19076,7 @@
         <v>45741</v>
       </c>
       <c r="AB99" t="s">
-        <v>45</v>
+        <v>3013</v>
       </c>
       <c r="AC99" t="s">
         <v>46</v>
@@ -19423,7 +19432,7 @@
         <v>45746</v>
       </c>
       <c r="AB103" t="s">
-        <v>45</v>
+        <v>2894</v>
       </c>
       <c r="AC103" t="s">
         <v>46</v>
@@ -19601,7 +19610,7 @@
         <v>45746</v>
       </c>
       <c r="AB105" t="s">
-        <v>45</v>
+        <v>3013</v>
       </c>
       <c r="AC105" t="s">
         <v>46</v>
@@ -19690,7 +19699,7 @@
         <v>45749</v>
       </c>
       <c r="AB106" t="s">
-        <v>45</v>
+        <v>3012</v>
       </c>
       <c r="AC106" t="s">
         <v>46</v>
@@ -19779,7 +19788,7 @@
         <v>45749</v>
       </c>
       <c r="AB107" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC107" t="s">
         <v>46</v>
@@ -20046,7 +20055,7 @@
         <v>45749</v>
       </c>
       <c r="AB110" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC110" t="s">
         <v>46</v>
@@ -22182,7 +22191,7 @@
         <v>45773</v>
       </c>
       <c r="AB134" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC134" t="s">
         <v>46</v>
@@ -22271,7 +22280,7 @@
         <v>45771</v>
       </c>
       <c r="AB135" t="s">
-        <v>45</v>
+        <v>3012</v>
       </c>
       <c r="AC135" t="s">
         <v>46</v>
@@ -22538,7 +22547,7 @@
         <v>45776</v>
       </c>
       <c r="AB138" t="s">
-        <v>45</v>
+        <v>3013</v>
       </c>
       <c r="AC138" t="s">
         <v>46</v>
@@ -22894,7 +22903,7 @@
         <v>45775</v>
       </c>
       <c r="AB142" t="s">
-        <v>45</v>
+        <v>2894</v>
       </c>
       <c r="AC142" t="s">
         <v>46</v>
@@ -23072,7 +23081,7 @@
         <v>45781</v>
       </c>
       <c r="AB144" t="s">
-        <v>45</v>
+        <v>3013</v>
       </c>
       <c r="AC144" t="s">
         <v>46</v>
@@ -23161,7 +23170,7 @@
         <v>45781</v>
       </c>
       <c r="AB145" t="s">
-        <v>45</v>
+        <v>3012</v>
       </c>
       <c r="AC145" t="s">
         <v>46</v>
@@ -23250,7 +23259,7 @@
         <v>45779</v>
       </c>
       <c r="AB146" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC146" t="s">
         <v>46</v>
@@ -23517,7 +23526,7 @@
         <v>45787</v>
       </c>
       <c r="AB149" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC149" t="s">
         <v>46</v>
@@ -25653,7 +25662,7 @@
         <v>45805</v>
       </c>
       <c r="AB173" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC173" t="s">
         <v>46</v>
@@ -25742,7 +25751,7 @@
         <v>45803</v>
       </c>
       <c r="AB174" t="s">
-        <v>45</v>
+        <v>3012</v>
       </c>
       <c r="AC174" t="s">
         <v>46</v>
@@ -26009,7 +26018,7 @@
         <v>45808</v>
       </c>
       <c r="AB177" t="s">
-        <v>45</v>
+        <v>3013</v>
       </c>
       <c r="AC177" t="s">
         <v>46</v>
@@ -26365,7 +26374,7 @@
         <v>45810</v>
       </c>
       <c r="AB181" t="s">
-        <v>45</v>
+        <v>2894</v>
       </c>
       <c r="AC181" t="s">
         <v>46</v>
@@ -26543,7 +26552,7 @@
         <v>45813</v>
       </c>
       <c r="AB183" t="s">
-        <v>45</v>
+        <v>3013</v>
       </c>
       <c r="AC183" t="s">
         <v>46</v>
@@ -26632,7 +26641,7 @@
         <v>45811</v>
       </c>
       <c r="AB184" t="s">
-        <v>45</v>
+        <v>3012</v>
       </c>
       <c r="AC184" t="s">
         <v>46</v>
@@ -26721,7 +26730,7 @@
         <v>45817</v>
       </c>
       <c r="AB185" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC185" t="s">
         <v>46</v>
@@ -26988,7 +26997,7 @@
         <v>45818</v>
       </c>
       <c r="AB188" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC188" t="s">
         <v>46</v>
@@ -29124,7 +29133,7 @@
         <v>45834</v>
       </c>
       <c r="AB212" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC212" t="s">
         <v>46</v>
@@ -29213,7 +29222,7 @@
         <v>45840</v>
       </c>
       <c r="AB213" t="s">
-        <v>45</v>
+        <v>3012</v>
       </c>
       <c r="AC213" t="s">
         <v>46</v>
@@ -29480,7 +29489,7 @@
         <v>45838</v>
       </c>
       <c r="AB216" t="s">
-        <v>45</v>
+        <v>3013</v>
       </c>
       <c r="AC216" t="s">
         <v>46</v>
@@ -29836,7 +29845,7 @@
         <v>45845</v>
       </c>
       <c r="AB220" t="s">
-        <v>45</v>
+        <v>2894</v>
       </c>
       <c r="AC220" t="s">
         <v>46</v>
@@ -30014,7 +30023,7 @@
         <v>45846</v>
       </c>
       <c r="AB222" t="s">
-        <v>45</v>
+        <v>3013</v>
       </c>
       <c r="AC222" t="s">
         <v>46</v>
@@ -30103,7 +30112,7 @@
         <v>45848</v>
       </c>
       <c r="AB223" t="s">
-        <v>45</v>
+        <v>3012</v>
       </c>
       <c r="AC223" t="s">
         <v>46</v>
@@ -30192,7 +30201,7 @@
         <v>45848</v>
       </c>
       <c r="AB224" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC224" t="s">
         <v>46</v>
@@ -30459,7 +30468,7 @@
         <v>45850</v>
       </c>
       <c r="AB227" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC227" t="s">
         <v>46</v>
@@ -32595,7 +32604,7 @@
         <v>45872</v>
       </c>
       <c r="AB251" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC251" t="s">
         <v>46</v>
@@ -32684,7 +32693,7 @@
         <v>45868</v>
       </c>
       <c r="AB252" t="s">
-        <v>45</v>
+        <v>3012</v>
       </c>
       <c r="AC252" t="s">
         <v>46</v>
@@ -32951,7 +32960,7 @@
         <v>45873</v>
       </c>
       <c r="AB255" t="s">
-        <v>45</v>
+        <v>3013</v>
       </c>
       <c r="AC255" t="s">
         <v>46</v>
@@ -33307,7 +33316,7 @@
         <v>45876</v>
       </c>
       <c r="AB259" t="s">
-        <v>45</v>
+        <v>2894</v>
       </c>
       <c r="AC259" t="s">
         <v>46</v>
@@ -33485,7 +33494,7 @@
         <v>45880</v>
       </c>
       <c r="AB261" t="s">
-        <v>45</v>
+        <v>3013</v>
       </c>
       <c r="AC261" t="s">
         <v>46</v>
@@ -33574,7 +33583,7 @@
         <v>45880</v>
       </c>
       <c r="AB262" t="s">
-        <v>45</v>
+        <v>3012</v>
       </c>
       <c r="AC262" t="s">
         <v>46</v>
@@ -33663,7 +33672,7 @@
         <v>45882</v>
       </c>
       <c r="AB263" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC263" t="s">
         <v>46</v>
@@ -33930,7 +33939,7 @@
         <v>45879</v>
       </c>
       <c r="AB266" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC266" t="s">
         <v>46</v>
@@ -36066,7 +36075,7 @@
         <v>45903</v>
       </c>
       <c r="AB290" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC290" t="s">
         <v>46</v>
@@ -36155,7 +36164,7 @@
         <v>45903</v>
       </c>
       <c r="AB291" t="s">
-        <v>45</v>
+        <v>3012</v>
       </c>
       <c r="AC291" t="s">
         <v>46</v>
@@ -36422,7 +36431,7 @@
         <v>45906</v>
       </c>
       <c r="AB294" t="s">
-        <v>45</v>
+        <v>3013</v>
       </c>
       <c r="AC294" t="s">
         <v>46</v>
@@ -36778,7 +36787,7 @@
         <v>45906</v>
       </c>
       <c r="AB298" t="s">
-        <v>45</v>
+        <v>2894</v>
       </c>
       <c r="AC298" t="s">
         <v>46</v>
@@ -36956,7 +36965,7 @@
         <v>45908</v>
       </c>
       <c r="AB300" t="s">
-        <v>45</v>
+        <v>3013</v>
       </c>
       <c r="AC300" t="s">
         <v>46</v>
@@ -37045,7 +37054,7 @@
         <v>45913</v>
       </c>
       <c r="AB301" t="s">
-        <v>45</v>
+        <v>3012</v>
       </c>
       <c r="AC301" t="s">
         <v>46</v>
@@ -37134,7 +37143,7 @@
         <v>45913</v>
       </c>
       <c r="AB302" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC302" t="s">
         <v>46</v>
@@ -37401,7 +37410,7 @@
         <v>45917</v>
       </c>
       <c r="AB305" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC305" t="s">
         <v>46</v>
@@ -39537,7 +39546,7 @@
         <v>45935</v>
       </c>
       <c r="AB329" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC329" t="s">
         <v>46</v>
@@ -39626,7 +39635,7 @@
         <v>45933</v>
       </c>
       <c r="AB330" t="s">
-        <v>45</v>
+        <v>3012</v>
       </c>
       <c r="AC330" t="s">
         <v>46</v>
@@ -39893,7 +39902,7 @@
         <v>45941</v>
       </c>
       <c r="AB333" t="s">
-        <v>45</v>
+        <v>3013</v>
       </c>
       <c r="AC333" t="s">
         <v>46</v>
@@ -40249,7 +40258,7 @@
         <v>45944</v>
       </c>
       <c r="AB337" t="s">
-        <v>45</v>
+        <v>2894</v>
       </c>
       <c r="AC337" t="s">
         <v>46</v>
@@ -40427,7 +40436,7 @@
         <v>45944</v>
       </c>
       <c r="AB339" t="s">
-        <v>45</v>
+        <v>3013</v>
       </c>
       <c r="AC339" t="s">
         <v>46</v>
@@ -40516,7 +40525,7 @@
         <v>45942</v>
       </c>
       <c r="AB340" t="s">
-        <v>45</v>
+        <v>3012</v>
       </c>
       <c r="AC340" t="s">
         <v>46</v>
@@ -40605,7 +40614,7 @@
         <v>45945</v>
       </c>
       <c r="AB341" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC341" t="s">
         <v>46</v>
@@ -40872,7 +40881,7 @@
         <v>45949</v>
       </c>
       <c r="AB344" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC344" t="s">
         <v>46</v>
@@ -43008,7 +43017,7 @@
         <v>45965</v>
       </c>
       <c r="AB368" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC368" t="s">
         <v>46</v>
@@ -43097,7 +43106,7 @@
         <v>45971</v>
       </c>
       <c r="AB369" t="s">
-        <v>45</v>
+        <v>3012</v>
       </c>
       <c r="AC369" t="s">
         <v>46</v>
@@ -43364,7 +43373,7 @@
         <v>45972</v>
       </c>
       <c r="AB372" t="s">
-        <v>45</v>
+        <v>3013</v>
       </c>
       <c r="AC372" t="s">
         <v>46</v>
@@ -43720,7 +43729,7 @@
         <v>45972</v>
       </c>
       <c r="AB376" t="s">
-        <v>45</v>
+        <v>2894</v>
       </c>
       <c r="AC376" t="s">
         <v>46</v>
@@ -43898,7 +43907,7 @@
         <v>45977</v>
       </c>
       <c r="AB378" t="s">
-        <v>45</v>
+        <v>3013</v>
       </c>
       <c r="AC378" t="s">
         <v>46</v>
@@ -43987,7 +43996,7 @@
         <v>45977</v>
       </c>
       <c r="AB379" t="s">
-        <v>45</v>
+        <v>3012</v>
       </c>
       <c r="AC379" t="s">
         <v>46</v>
@@ -44076,7 +44085,7 @@
         <v>45975</v>
       </c>
       <c r="AB380" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC380" t="s">
         <v>46</v>
@@ -44343,7 +44352,7 @@
         <v>45980</v>
       </c>
       <c r="AB383" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC383" t="s">
         <v>46</v>
@@ -46479,7 +46488,7 @@
         <v>46002</v>
       </c>
       <c r="AB407" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC407" t="s">
         <v>46</v>
@@ -46568,7 +46577,7 @@
         <v>46002</v>
       </c>
       <c r="AB408" t="s">
-        <v>45</v>
+        <v>3012</v>
       </c>
       <c r="AC408" t="s">
         <v>46</v>
@@ -46835,7 +46844,7 @@
         <v>46002</v>
       </c>
       <c r="AB411" t="s">
-        <v>45</v>
+        <v>3013</v>
       </c>
       <c r="AC411" t="s">
         <v>46</v>
@@ -47191,7 +47200,7 @@
         <v>46007</v>
       </c>
       <c r="AB415" t="s">
-        <v>45</v>
+        <v>2894</v>
       </c>
       <c r="AC415" t="s">
         <v>46</v>
@@ -47369,7 +47378,7 @@
         <v>46007</v>
       </c>
       <c r="AB417" t="s">
-        <v>45</v>
+        <v>3013</v>
       </c>
       <c r="AC417" t="s">
         <v>46</v>
@@ -47458,7 +47467,7 @@
         <v>46006</v>
       </c>
       <c r="AB418" t="s">
-        <v>45</v>
+        <v>3012</v>
       </c>
       <c r="AC418" t="s">
         <v>46</v>
@@ -47547,7 +47556,7 @@
         <v>46012</v>
       </c>
       <c r="AB419" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC419" t="s">
         <v>46</v>
@@ -47814,7 +47823,7 @@
         <v>46010</v>
       </c>
       <c r="AB422" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC422" t="s">
         <v>46</v>
@@ -49950,7 +49959,7 @@
         <v>46034</v>
       </c>
       <c r="AB446" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC446" t="s">
         <v>46</v>
@@ -50039,7 +50048,7 @@
         <v>46034</v>
       </c>
       <c r="AB447" t="s">
-        <v>45</v>
+        <v>3012</v>
       </c>
       <c r="AC447" t="s">
         <v>46</v>
@@ -50306,7 +50315,7 @@
         <v>46033</v>
       </c>
       <c r="AB450" t="s">
-        <v>45</v>
+        <v>3013</v>
       </c>
       <c r="AC450" t="s">
         <v>46</v>
@@ -50662,7 +50671,7 @@
         <v>46037</v>
       </c>
       <c r="AB454" t="s">
-        <v>45</v>
+        <v>2894</v>
       </c>
       <c r="AC454" t="s">
         <v>46</v>
@@ -50840,7 +50849,7 @@
         <v>46038</v>
       </c>
       <c r="AB456" t="s">
-        <v>45</v>
+        <v>3013</v>
       </c>
       <c r="AC456" t="s">
         <v>46</v>
@@ -50929,7 +50938,7 @@
         <v>46044</v>
       </c>
       <c r="AB457" t="s">
-        <v>45</v>
+        <v>3012</v>
       </c>
       <c r="AC457" t="s">
         <v>46</v>
@@ -51018,7 +51027,7 @@
         <v>46044</v>
       </c>
       <c r="AB458" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC458" t="s">
         <v>46</v>
@@ -51285,7 +51294,7 @@
         <v>46044</v>
       </c>
       <c r="AB461" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC461" t="s">
         <v>46</v>
@@ -53421,7 +53430,7 @@
         <v>46064</v>
       </c>
       <c r="AB485" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC485" t="s">
         <v>46</v>
@@ -53510,7 +53519,7 @@
         <v>46067</v>
       </c>
       <c r="AB486" t="s">
-        <v>45</v>
+        <v>3012</v>
       </c>
       <c r="AC486" t="s">
         <v>46</v>
@@ -53777,7 +53786,7 @@
         <v>46071</v>
       </c>
       <c r="AB489" t="s">
-        <v>45</v>
+        <v>3013</v>
       </c>
       <c r="AC489" t="s">
         <v>46</v>
@@ -54133,7 +54142,7 @@
         <v>46074</v>
       </c>
       <c r="AB493" t="s">
-        <v>45</v>
+        <v>2894</v>
       </c>
       <c r="AC493" t="s">
         <v>46</v>
@@ -54311,7 +54320,7 @@
         <v>46076</v>
       </c>
       <c r="AB495" t="s">
-        <v>45</v>
+        <v>3013</v>
       </c>
       <c r="AC495" t="s">
         <v>46</v>
@@ -54400,7 +54409,7 @@
         <v>46076</v>
       </c>
       <c r="AB496" t="s">
-        <v>45</v>
+        <v>3012</v>
       </c>
       <c r="AC496" t="s">
         <v>46</v>
@@ -54489,7 +54498,7 @@
         <v>46074</v>
       </c>
       <c r="AB497" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC497" t="s">
         <v>46</v>
@@ -54756,7 +54765,7 @@
         <v>46079</v>
       </c>
       <c r="AB500" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC500" t="s">
         <v>46</v>
@@ -56892,7 +56901,7 @@
         <v>46095</v>
       </c>
       <c r="AB524" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC524" t="s">
         <v>46</v>
@@ -56981,7 +56990,7 @@
         <v>46098</v>
       </c>
       <c r="AB525" t="s">
-        <v>45</v>
+        <v>3012</v>
       </c>
       <c r="AC525" t="s">
         <v>46</v>
@@ -57248,7 +57257,7 @@
         <v>46102</v>
       </c>
       <c r="AB528" t="s">
-        <v>45</v>
+        <v>3013</v>
       </c>
       <c r="AC528" t="s">
         <v>46</v>
@@ -57604,7 +57613,7 @@
         <v>46101</v>
       </c>
       <c r="AB532" t="s">
-        <v>45</v>
+        <v>2894</v>
       </c>
       <c r="AC532" t="s">
         <v>46</v>
@@ -57782,7 +57791,7 @@
         <v>46107</v>
       </c>
       <c r="AB534" t="s">
-        <v>45</v>
+        <v>3013</v>
       </c>
       <c r="AC534" t="s">
         <v>46</v>
@@ -57871,7 +57880,7 @@
         <v>46107</v>
       </c>
       <c r="AB535" t="s">
-        <v>45</v>
+        <v>3012</v>
       </c>
       <c r="AC535" t="s">
         <v>46</v>
@@ -57960,7 +57969,7 @@
         <v>46108</v>
       </c>
       <c r="AB536" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC536" t="s">
         <v>46</v>
@@ -58227,7 +58236,7 @@
         <v>46110</v>
       </c>
       <c r="AB539" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC539" t="s">
         <v>46</v>
@@ -63834,7 +63843,7 @@
         <v>46160</v>
       </c>
       <c r="AB602" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC602" t="s">
         <v>46</v>
@@ -63923,7 +63932,7 @@
         <v>46166</v>
       </c>
       <c r="AB603" t="s">
-        <v>45</v>
+        <v>3012</v>
       </c>
       <c r="AC603" t="s">
         <v>46</v>
@@ -64190,7 +64199,7 @@
         <v>46167</v>
       </c>
       <c r="AB606" t="s">
-        <v>45</v>
+        <v>3013</v>
       </c>
       <c r="AC606" t="s">
         <v>46</v>
@@ -64546,7 +64555,7 @@
         <v>46171</v>
       </c>
       <c r="AB610" t="s">
-        <v>45</v>
+        <v>2894</v>
       </c>
       <c r="AC610" t="s">
         <v>46</v>
@@ -64724,7 +64733,7 @@
         <v>46172</v>
       </c>
       <c r="AB612" t="s">
-        <v>45</v>
+        <v>3013</v>
       </c>
       <c r="AC612" t="s">
         <v>46</v>
@@ -64813,7 +64822,7 @@
         <v>46174</v>
       </c>
       <c r="AB613" t="s">
-        <v>45</v>
+        <v>3012</v>
       </c>
       <c r="AC613" t="s">
         <v>46</v>
@@ -64902,7 +64911,7 @@
         <v>46174</v>
       </c>
       <c r="AB614" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC614" t="s">
         <v>46</v>
@@ -65169,7 +65178,7 @@
         <v>46176</v>
       </c>
       <c r="AB617" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC617" t="s">
         <v>46</v>
@@ -70776,7 +70785,7 @@
         <v>46229</v>
       </c>
       <c r="AB680" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC680" t="s">
         <v>46</v>
@@ -70865,7 +70874,7 @@
         <v>46229</v>
       </c>
       <c r="AB681" t="s">
-        <v>45</v>
+        <v>3012</v>
       </c>
       <c r="AC681" t="s">
         <v>46</v>
@@ -71132,7 +71141,7 @@
         <v>46232</v>
       </c>
       <c r="AB684" t="s">
-        <v>45</v>
+        <v>3013</v>
       </c>
       <c r="AC684" t="s">
         <v>46</v>
@@ -71488,7 +71497,7 @@
         <v>46232</v>
       </c>
       <c r="AB688" t="s">
-        <v>45</v>
+        <v>2894</v>
       </c>
       <c r="AC688" t="s">
         <v>46</v>
@@ -71666,7 +71675,7 @@
         <v>46237</v>
       </c>
       <c r="AB690" t="s">
-        <v>45</v>
+        <v>3013</v>
       </c>
       <c r="AC690" t="s">
         <v>46</v>
@@ -71755,7 +71764,7 @@
         <v>46237</v>
       </c>
       <c r="AB691" t="s">
-        <v>45</v>
+        <v>3012</v>
       </c>
       <c r="AC691" t="s">
         <v>46</v>
@@ -71844,7 +71853,7 @@
         <v>46235</v>
       </c>
       <c r="AB692" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC692" t="s">
         <v>46</v>
@@ -72111,7 +72120,7 @@
         <v>46239</v>
       </c>
       <c r="AB695" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC695" t="s">
         <v>46</v>
@@ -77718,7 +77727,7 @@
         <v>46290</v>
       </c>
       <c r="AB758" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC758" t="s">
         <v>46</v>
@@ -77807,7 +77816,7 @@
         <v>46296</v>
       </c>
       <c r="AB759" t="s">
-        <v>45</v>
+        <v>3012</v>
       </c>
       <c r="AC759" t="s">
         <v>46</v>
@@ -78074,7 +78083,7 @@
         <v>46293</v>
       </c>
       <c r="AB762" t="s">
-        <v>45</v>
+        <v>3013</v>
       </c>
       <c r="AC762" t="s">
         <v>46</v>
@@ -78430,7 +78439,7 @@
         <v>46301</v>
       </c>
       <c r="AB766" t="s">
-        <v>45</v>
+        <v>2894</v>
       </c>
       <c r="AC766" t="s">
         <v>46</v>
@@ -78608,7 +78617,7 @@
         <v>46299</v>
       </c>
       <c r="AB768" t="s">
-        <v>45</v>
+        <v>3013</v>
       </c>
       <c r="AC768" t="s">
         <v>46</v>
@@ -78697,7 +78706,7 @@
         <v>46305</v>
       </c>
       <c r="AB769" t="s">
-        <v>45</v>
+        <v>3012</v>
       </c>
       <c r="AC769" t="s">
         <v>46</v>
@@ -78786,7 +78795,7 @@
         <v>46305</v>
       </c>
       <c r="AB770" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC770" t="s">
         <v>46</v>
@@ -79053,7 +79062,7 @@
         <v>46306</v>
       </c>
       <c r="AB773" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC773" t="s">
         <v>46</v>
@@ -84660,7 +84669,7 @@
         <v>46360</v>
       </c>
       <c r="AB836" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC836" t="s">
         <v>46</v>
@@ -84749,7 +84758,7 @@
         <v>46358</v>
       </c>
       <c r="AB837" t="s">
-        <v>45</v>
+        <v>3012</v>
       </c>
       <c r="AC837" t="s">
         <v>46</v>
@@ -85016,7 +85025,7 @@
         <v>46359</v>
       </c>
       <c r="AB840" t="s">
-        <v>45</v>
+        <v>3013</v>
       </c>
       <c r="AC840" t="s">
         <v>46</v>
@@ -85372,7 +85381,7 @@
         <v>46362</v>
       </c>
       <c r="AB844" t="s">
-        <v>45</v>
+        <v>2894</v>
       </c>
       <c r="AC844" t="s">
         <v>46</v>
@@ -85550,7 +85559,7 @@
         <v>46368</v>
       </c>
       <c r="AB846" t="s">
-        <v>45</v>
+        <v>3013</v>
       </c>
       <c r="AC846" t="s">
         <v>46</v>
@@ -85639,7 +85648,7 @@
         <v>46368</v>
       </c>
       <c r="AB847" t="s">
-        <v>45</v>
+        <v>3012</v>
       </c>
       <c r="AC847" t="s">
         <v>46</v>
@@ -85728,7 +85737,7 @@
         <v>46366</v>
       </c>
       <c r="AB848" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC848" t="s">
         <v>46</v>
@@ -85995,7 +86004,7 @@
         <v>46373</v>
       </c>
       <c r="AB851" t="s">
-        <v>45</v>
+        <v>3011</v>
       </c>
       <c r="AC851" t="s">
         <v>46</v>

</xml_diff>